<commit_message>
Updated Land-use file using Indonesia Data
</commit_message>
<xml_diff>
--- a/InputData/land/CApULAbIFM/CO2 Abated per Unit Land Area by Impr For Mgmt.xlsx
+++ b/InputData/land/CApULAbIFM/CO2 Abated per Unit Land Area by Impr For Mgmt.xlsx
@@ -1,38 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25028"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\land\CApULAbIFM\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF08A53-F280-4704-83EC-0E3DACD573C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="320" yWindow="320" windowWidth="18820" windowHeight="6560"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="CApULAbIFM" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>CApULAbIFM CO2 Abated per Unit Land Area by Improved Forest Management</t>
   </si>
@@ -40,19 +23,25 @@
     <t>Source:</t>
   </si>
   <si>
+    <t>none needed</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>We do not use the Improved Forest Management policy in the Indonesia model.</t>
+  </si>
+  <si>
     <t>CO2 Abated (g)</t>
   </si>
   <si>
     <t>Per Acre</t>
-  </si>
-  <si>
-    <t>consultation with American Forest Foundation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -90,14 +79,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -107,9 +94,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -158,7 +142,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -191,26 +175,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -243,23 +210,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -435,55 +385,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-    </row>
-    <row r="6" spans="1:2" ht="14.45" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="15.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3">
-        <f>1.5*10^6</f>
-        <v>1500000</v>
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated with the firts version
</commit_message>
<xml_diff>
--- a/InputData/land/CApULAbIFM/CO2 Abated per Unit Land Area by Impr For Mgmt.xlsx
+++ b/InputData/land/CApULAbIFM/CO2 Abated per Unit Land Area by Impr For Mgmt.xlsx
@@ -1,21 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25028"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\land\CApULAbIFM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF08A53-F280-4704-83EC-0E3DACD573C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="320" windowWidth="18820" windowHeight="6560"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="CApULAbIFM" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>CApULAbIFM CO2 Abated per Unit Land Area by Improved Forest Management</t>
   </si>
@@ -23,25 +40,19 @@
     <t>Source:</t>
   </si>
   <si>
-    <t>none needed</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>We do not use the Improved Forest Management policy in the Indonesia model.</t>
-  </si>
-  <si>
     <t>CO2 Abated (g)</t>
   </si>
   <si>
     <t>Per Acre</t>
   </si>
+  <si>
+    <t>consultation with American Forest Foundation</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -79,12 +90,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -94,6 +107,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -142,7 +158,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -175,9 +191,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -210,6 +243,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -385,60 +435,55 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="14.45" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
+    <row r="6" spans="1:2" ht="14.45" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="B2" s="3">
+        <f>1.5*10^6</f>
+        <v>1500000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>